<commit_message>
Use cleaned data in pipeline
</commit_message>
<xml_diff>
--- a/clarity-pipeline/src/test/resources/evaluation/12_14_2025.xlsx
+++ b/clarity-pipeline/src/test/resources/evaluation/12_14_2025.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="48">
   <si>
     <t>Name</t>
   </si>
@@ -36,6 +36,30 @@
   </si>
   <si>
     <t>GPT 5.2</t>
+  </si>
+  <si>
+    <t>reasoning-effort-auto:cleaned:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-auto:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-none:cleaned:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-high:cleaned:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-none:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-high:cleaned:evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-none:cleaned:evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>reasoning-effort-auto:cleaned:evasion-based:single:few-shot:v1</t>
   </si>
   <si>
     <t>rag:reasoning-effort-auto:evasion-based:single:few-shot:v1</t>
@@ -214,11 +238,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="14.95703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="47.984375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="57.91015625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="9.015625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="9.15625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="6.30859375" customWidth="true" bestFit="true"/>
@@ -257,19 +281,19 @@
         <v>8</v>
       </c>
       <c r="C2" t="n" s="3">
-        <v>0.808</v>
+        <v>0.818</v>
       </c>
       <c r="D2" t="n" s="3">
-        <v>0.78</v>
+        <v>0.794</v>
       </c>
       <c r="E2" t="n" s="3">
-        <v>0.749</v>
+        <v>0.764</v>
       </c>
       <c r="F2" t="n" s="3">
-        <v>0.763</v>
+        <v>0.776</v>
       </c>
       <c r="G2" t="n" s="3">
-        <v>0.808</v>
+        <v>0.818</v>
       </c>
     </row>
     <row r="3">
@@ -280,19 +304,19 @@
         <v>9</v>
       </c>
       <c r="C3" t="n" s="3">
-        <v>0.802</v>
+        <v>0.815</v>
       </c>
       <c r="D3" t="n" s="3">
-        <v>0.792</v>
+        <v>0.818</v>
       </c>
       <c r="E3" t="n" s="3">
-        <v>0.689</v>
+        <v>0.763</v>
       </c>
       <c r="F3" t="n" s="3">
-        <v>0.727</v>
+        <v>0.787</v>
       </c>
       <c r="G3" t="n" s="3">
-        <v>0.802</v>
+        <v>0.815</v>
       </c>
     </row>
     <row r="4">
@@ -303,19 +327,19 @@
         <v>10</v>
       </c>
       <c r="C4" t="n" s="3">
-        <v>0.815</v>
+        <v>0.805</v>
       </c>
       <c r="D4" t="n" s="3">
-        <v>0.806</v>
+        <v>0.783</v>
       </c>
       <c r="E4" t="n" s="3">
-        <v>0.752</v>
+        <v>0.745</v>
       </c>
       <c r="F4" t="n" s="3">
-        <v>0.776</v>
+        <v>0.758</v>
       </c>
       <c r="G4" t="n" s="3">
-        <v>0.815</v>
+        <v>0.805</v>
       </c>
     </row>
     <row r="5">
@@ -326,249 +350,249 @@
         <v>11</v>
       </c>
       <c r="C5" t="n" s="3">
-        <v>0.831</v>
+        <v>0.75</v>
       </c>
       <c r="D5" t="n" s="3">
-        <v>0.865</v>
+        <v>0.722</v>
       </c>
       <c r="E5" t="n" s="3">
-        <v>0.724</v>
+        <v>0.8</v>
       </c>
       <c r="F5" t="n" s="3">
-        <v>0.776</v>
+        <v>0.746</v>
       </c>
       <c r="G5" t="n" s="3">
-        <v>0.831</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B6" t="s" s="2">
-        <v>13</v>
-      </c>
       <c r="C6" t="n" s="3">
-        <v>0.575</v>
+        <v>0.808</v>
       </c>
       <c r="D6" t="n" s="3">
-        <v>0.514</v>
+        <v>0.775</v>
       </c>
       <c r="E6" t="n" s="3">
-        <v>0.633</v>
+        <v>0.744</v>
       </c>
       <c r="F6" t="n" s="3">
-        <v>0.519</v>
+        <v>0.759</v>
       </c>
       <c r="G6" t="n" s="3">
-        <v>0.575</v>
+        <v>0.808</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" t="n" s="3">
-        <v>0.75</v>
+        <v>0.763</v>
       </c>
       <c r="D7" t="n" s="3">
-        <v>0.71</v>
+        <v>0.702</v>
       </c>
       <c r="E7" t="n" s="3">
-        <v>0.637</v>
+        <v>0.791</v>
       </c>
       <c r="F7" t="n" s="3">
-        <v>0.659</v>
+        <v>0.737</v>
       </c>
       <c r="G7" t="n" s="3">
-        <v>0.75</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="n" s="3">
-        <v>0.705</v>
+        <v>0.799</v>
       </c>
       <c r="D8" t="n" s="3">
-        <v>0.611</v>
+        <v>0.802</v>
       </c>
       <c r="E8" t="n" s="3">
-        <v>0.651</v>
+        <v>0.718</v>
       </c>
       <c r="F8" t="n" s="3">
-        <v>0.609</v>
+        <v>0.749</v>
       </c>
       <c r="G8" t="n" s="3">
-        <v>0.705</v>
+        <v>0.799</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n" s="3">
-        <v>0.786</v>
+        <v>0.805</v>
       </c>
       <c r="D9" t="n" s="3">
-        <v>0.776</v>
+        <v>0.798</v>
       </c>
       <c r="E9" t="n" s="3">
-        <v>0.658</v>
+        <v>0.706</v>
       </c>
       <c r="F9" t="n" s="3">
-        <v>0.699</v>
+        <v>0.734</v>
       </c>
       <c r="G9" t="n" s="3">
-        <v>0.786</v>
+        <v>0.805</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="B10" t="s" s="2">
-        <v>15</v>
-      </c>
       <c r="C10" t="n" s="3">
-        <v>0.773</v>
+        <v>0.808</v>
       </c>
       <c r="D10" t="n" s="3">
-        <v>0.776</v>
+        <v>0.78</v>
       </c>
       <c r="E10" t="n" s="3">
-        <v>0.649</v>
+        <v>0.749</v>
       </c>
       <c r="F10" t="n" s="3">
-        <v>0.689</v>
+        <v>0.763</v>
       </c>
       <c r="G10" t="n" s="3">
-        <v>0.773</v>
+        <v>0.808</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="B11" t="s" s="2">
-        <v>14</v>
-      </c>
       <c r="C11" t="n" s="3">
-        <v>0.731</v>
+        <v>0.802</v>
       </c>
       <c r="D11" t="n" s="3">
-        <v>0.692</v>
+        <v>0.792</v>
       </c>
       <c r="E11" t="n" s="3">
-        <v>0.796</v>
+        <v>0.689</v>
       </c>
       <c r="F11" t="n" s="3">
-        <v>0.726</v>
+        <v>0.727</v>
       </c>
       <c r="G11" t="n" s="3">
-        <v>0.731</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C12" t="n" s="3">
-        <v>0.636</v>
+        <v>0.815</v>
       </c>
       <c r="D12" t="n" s="3">
-        <v>0.585</v>
+        <v>0.806</v>
       </c>
       <c r="E12" t="n" s="3">
-        <v>0.746</v>
+        <v>0.752</v>
       </c>
       <c r="F12" t="n" s="3">
-        <v>0.613</v>
+        <v>0.776</v>
       </c>
       <c r="G12" t="n" s="3">
-        <v>0.636</v>
+        <v>0.815</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="n" s="3">
-        <v>0.679</v>
+        <v>0.831</v>
       </c>
       <c r="D13" t="n" s="3">
-        <v>0.619</v>
+        <v>0.865</v>
       </c>
       <c r="E13" t="n" s="3">
-        <v>0.765</v>
+        <v>0.724</v>
       </c>
       <c r="F13" t="n" s="3">
-        <v>0.65</v>
+        <v>0.776</v>
       </c>
       <c r="G13" t="n" s="3">
-        <v>0.679</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C14" t="n" s="3">
-        <v>0.812</v>
+        <v>0.575</v>
       </c>
       <c r="D14" t="n" s="3">
-        <v>0.826</v>
+        <v>0.514</v>
       </c>
       <c r="E14" t="n" s="3">
-        <v>0.717</v>
+        <v>0.633</v>
       </c>
       <c r="F14" t="n" s="3">
-        <v>0.758</v>
+        <v>0.519</v>
       </c>
       <c r="G14" t="n" s="3">
-        <v>0.812</v>
+        <v>0.575</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C15" t="n" s="3">
-        <v>0.695</v>
+        <v>0.75</v>
       </c>
       <c r="D15" t="n" s="3">
-        <v>0.636</v>
+        <v>0.71</v>
       </c>
       <c r="E15" t="n" s="3">
-        <v>0.666</v>
+        <v>0.637</v>
       </c>
       <c r="F15" t="n" s="3">
-        <v>0.599</v>
+        <v>0.659</v>
       </c>
       <c r="G15" t="n" s="3">
-        <v>0.695</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="16">
@@ -576,617 +600,617 @@
         <v>20</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C16" t="n" s="3">
-        <v>0.753</v>
+        <v>0.705</v>
       </c>
       <c r="D16" t="n" s="3">
-        <v>0.856</v>
+        <v>0.611</v>
       </c>
       <c r="E16" t="n" s="3">
-        <v>0.595</v>
+        <v>0.651</v>
       </c>
       <c r="F16" t="n" s="3">
-        <v>0.636</v>
+        <v>0.609</v>
       </c>
       <c r="G16" t="n" s="3">
-        <v>0.753</v>
+        <v>0.705</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s" s="2">
         <v>22</v>
       </c>
       <c r="C17" t="n" s="3">
-        <v>0.685</v>
+        <v>0.786</v>
       </c>
       <c r="D17" t="n" s="3">
-        <v>0.664</v>
+        <v>0.776</v>
       </c>
       <c r="E17" t="n" s="3">
-        <v>0.575</v>
+        <v>0.658</v>
       </c>
       <c r="F17" t="n" s="3">
-        <v>0.588</v>
+        <v>0.699</v>
       </c>
       <c r="G17" t="n" s="3">
-        <v>0.685</v>
+        <v>0.786</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B18" t="s" s="2">
         <v>23</v>
       </c>
       <c r="C18" t="n" s="3">
-        <v>0.76</v>
+        <v>0.773</v>
       </c>
       <c r="D18" t="n" s="3">
-        <v>0.784</v>
+        <v>0.776</v>
       </c>
       <c r="E18" t="n" s="3">
-        <v>0.542</v>
+        <v>0.649</v>
       </c>
       <c r="F18" t="n" s="3">
-        <v>0.593</v>
+        <v>0.689</v>
       </c>
       <c r="G18" t="n" s="3">
-        <v>0.76</v>
+        <v>0.773</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C19" t="n" s="3">
-        <v>0.747</v>
+        <v>0.731</v>
       </c>
       <c r="D19" t="n" s="3">
-        <v>0.72</v>
+        <v>0.692</v>
       </c>
       <c r="E19" t="n" s="3">
-        <v>0.595</v>
+        <v>0.796</v>
       </c>
       <c r="F19" t="n" s="3">
-        <v>0.636</v>
+        <v>0.726</v>
       </c>
       <c r="G19" t="n" s="3">
-        <v>0.747</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C20" t="n" s="3">
-        <v>0.782</v>
+        <v>0.636</v>
       </c>
       <c r="D20" t="n" s="3">
-        <v>0.804</v>
+        <v>0.585</v>
       </c>
       <c r="E20" t="n" s="3">
-        <v>0.664</v>
+        <v>0.746</v>
       </c>
       <c r="F20" t="n" s="3">
-        <v>0.692</v>
+        <v>0.613</v>
       </c>
       <c r="G20" t="n" s="3">
-        <v>0.782</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s" s="2">
         <v>26</v>
       </c>
       <c r="C21" t="n" s="3">
-        <v>0.731</v>
+        <v>0.679</v>
       </c>
       <c r="D21" t="n" s="3">
-        <v>0.756</v>
+        <v>0.619</v>
       </c>
       <c r="E21" t="n" s="3">
-        <v>0.558</v>
+        <v>0.765</v>
       </c>
       <c r="F21" t="n" s="3">
-        <v>0.591</v>
+        <v>0.65</v>
       </c>
       <c r="G21" t="n" s="3">
-        <v>0.731</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C22" t="n" s="3">
-        <v>0.769</v>
+        <v>0.812</v>
       </c>
       <c r="D22" t="n" s="3">
-        <v>0.783</v>
+        <v>0.826</v>
       </c>
       <c r="E22" t="n" s="3">
-        <v>0.629</v>
+        <v>0.717</v>
       </c>
       <c r="F22" t="n" s="3">
-        <v>0.663</v>
+        <v>0.758</v>
       </c>
       <c r="G22" t="n" s="3">
-        <v>0.769</v>
+        <v>0.812</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C23" t="n" s="3">
-        <v>0.737</v>
+        <v>0.695</v>
       </c>
       <c r="D23" t="n" s="3">
-        <v>0.772</v>
+        <v>0.636</v>
       </c>
       <c r="E23" t="n" s="3">
-        <v>0.563</v>
+        <v>0.666</v>
       </c>
       <c r="F23" t="n" s="3">
         <v>0.599</v>
       </c>
       <c r="G23" t="n" s="3">
-        <v>0.737</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C24" t="n" s="3">
-        <v>0.731</v>
+        <v>0.753</v>
       </c>
       <c r="D24" t="n" s="3">
-        <v>0.673</v>
+        <v>0.856</v>
       </c>
       <c r="E24" t="n" s="3">
-        <v>0.599</v>
+        <v>0.595</v>
       </c>
       <c r="F24" t="n" s="3">
-        <v>0.601</v>
+        <v>0.636</v>
       </c>
       <c r="G24" t="n" s="3">
-        <v>0.731</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C25" t="n" s="3">
-        <v>0.753</v>
+        <v>0.685</v>
       </c>
       <c r="D25" t="n" s="3">
-        <v>0.867</v>
+        <v>0.664</v>
       </c>
       <c r="E25" t="n" s="3">
-        <v>0.602</v>
+        <v>0.575</v>
       </c>
       <c r="F25" t="n" s="3">
-        <v>0.636</v>
+        <v>0.588</v>
       </c>
       <c r="G25" t="n" s="3">
-        <v>0.753</v>
+        <v>0.685</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C26" t="n" s="3">
-        <v>0.695</v>
+        <v>0.76</v>
       </c>
       <c r="D26" t="n" s="3">
-        <v>0.637</v>
+        <v>0.784</v>
       </c>
       <c r="E26" t="n" s="3">
-        <v>0.602</v>
+        <v>0.542</v>
       </c>
       <c r="F26" t="n" s="3">
-        <v>0.553</v>
+        <v>0.593</v>
       </c>
       <c r="G26" t="n" s="3">
-        <v>0.695</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C27" t="n" s="3">
-        <v>0.708</v>
+        <v>0.747</v>
       </c>
       <c r="D27" t="n" s="3">
-        <v>0.682</v>
+        <v>0.72</v>
       </c>
       <c r="E27" t="n" s="3">
-        <v>0.655</v>
+        <v>0.595</v>
       </c>
       <c r="F27" t="n" s="3">
-        <v>0.663</v>
+        <v>0.636</v>
       </c>
       <c r="G27" t="n" s="3">
-        <v>0.708</v>
+        <v>0.747</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C28" t="n" s="3">
-        <v>0.744</v>
+        <v>0.782</v>
       </c>
       <c r="D28" t="n" s="3">
-        <v>0.728</v>
+        <v>0.804</v>
       </c>
       <c r="E28" t="n" s="3">
-        <v>0.707</v>
+        <v>0.664</v>
       </c>
       <c r="F28" t="n" s="3">
-        <v>0.708</v>
+        <v>0.692</v>
       </c>
       <c r="G28" t="n" s="3">
-        <v>0.744</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C29" t="n" s="3">
-        <v>0.772</v>
+        <v>0.731</v>
       </c>
       <c r="D29" t="n" s="3">
-        <v>0.755</v>
+        <v>0.756</v>
       </c>
       <c r="E29" t="n" s="3">
-        <v>0.759</v>
+        <v>0.558</v>
       </c>
       <c r="F29" t="n" s="3">
-        <v>0.752</v>
+        <v>0.591</v>
       </c>
       <c r="G29" t="n" s="3">
-        <v>0.772</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C30" t="n" s="3">
-        <v>0.782</v>
+        <v>0.769</v>
       </c>
       <c r="D30" t="n" s="3">
-        <v>0.745</v>
+        <v>0.783</v>
       </c>
       <c r="E30" t="n" s="3">
-        <v>0.76</v>
+        <v>0.629</v>
       </c>
       <c r="F30" t="n" s="3">
-        <v>0.752</v>
+        <v>0.663</v>
       </c>
       <c r="G30" t="n" s="3">
-        <v>0.782</v>
+        <v>0.769</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C31" t="n" s="3">
-        <v>0.763</v>
+        <v>0.737</v>
       </c>
       <c r="D31" t="n" s="3">
-        <v>0.753</v>
+        <v>0.772</v>
       </c>
       <c r="E31" t="n" s="3">
-        <v>0.709</v>
+        <v>0.563</v>
       </c>
       <c r="F31" t="n" s="3">
-        <v>0.723</v>
+        <v>0.599</v>
       </c>
       <c r="G31" t="n" s="3">
-        <v>0.763</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C32" t="n" s="3">
-        <v>0.688</v>
+        <v>0.731</v>
       </c>
       <c r="D32" t="n" s="3">
-        <v>0.6</v>
+        <v>0.673</v>
       </c>
       <c r="E32" t="n" s="3">
-        <v>0.669</v>
+        <v>0.599</v>
       </c>
       <c r="F32" t="n" s="3">
-        <v>0.622</v>
+        <v>0.601</v>
       </c>
       <c r="G32" t="n" s="3">
-        <v>0.688</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C33" t="n" s="3">
-        <v>0.75</v>
+        <v>0.753</v>
       </c>
       <c r="D33" t="n" s="3">
-        <v>0.711</v>
+        <v>0.867</v>
       </c>
       <c r="E33" t="n" s="3">
-        <v>0.748</v>
+        <v>0.602</v>
       </c>
       <c r="F33" t="n" s="3">
-        <v>0.728</v>
+        <v>0.636</v>
       </c>
       <c r="G33" t="n" s="3">
-        <v>0.75</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C34" t="n" s="3">
-        <v>0.763</v>
+        <v>0.695</v>
       </c>
       <c r="D34" t="n" s="3">
-        <v>0.725</v>
+        <v>0.637</v>
       </c>
       <c r="E34" t="n" s="3">
-        <v>0.701</v>
+        <v>0.602</v>
       </c>
       <c r="F34" t="n" s="3">
-        <v>0.707</v>
+        <v>0.553</v>
       </c>
       <c r="G34" t="n" s="3">
-        <v>0.763</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="B35" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="B35" t="s" s="2">
-        <v>32</v>
-      </c>
       <c r="C35" t="n" s="3">
-        <v>0.747</v>
+        <v>0.708</v>
       </c>
       <c r="D35" t="n" s="3">
-        <v>0.674</v>
+        <v>0.682</v>
       </c>
       <c r="E35" t="n" s="3">
-        <v>0.739</v>
+        <v>0.655</v>
       </c>
       <c r="F35" t="n" s="3">
-        <v>0.701</v>
+        <v>0.663</v>
       </c>
       <c r="G35" t="n" s="3">
-        <v>0.747</v>
+        <v>0.708</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="C36" t="n" s="3">
+        <v>0.744</v>
+      </c>
+      <c r="D36" t="n" s="3">
+        <v>0.728</v>
+      </c>
+      <c r="E36" t="n" s="3">
+        <v>0.707</v>
+      </c>
+      <c r="F36" t="n" s="3">
         <v>0.708</v>
       </c>
-      <c r="D36" t="n" s="3">
-        <v>0.618</v>
-      </c>
-      <c r="E36" t="n" s="3">
-        <v>0.738</v>
-      </c>
-      <c r="F36" t="n" s="3">
-        <v>0.651</v>
-      </c>
       <c r="G36" t="n" s="3">
-        <v>0.708</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C37" t="n" s="3">
-        <v>0.662</v>
+        <v>0.772</v>
       </c>
       <c r="D37" t="n" s="3">
-        <v>0.638</v>
+        <v>0.755</v>
       </c>
       <c r="E37" t="n" s="3">
-        <v>0.741</v>
+        <v>0.759</v>
       </c>
       <c r="F37" t="n" s="3">
-        <v>0.652</v>
+        <v>0.752</v>
       </c>
       <c r="G37" t="n" s="3">
-        <v>0.662</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C38" t="n" s="3">
-        <v>0.679</v>
+        <v>0.782</v>
       </c>
       <c r="D38" t="n" s="3">
-        <v>0.657</v>
+        <v>0.745</v>
       </c>
       <c r="E38" t="n" s="3">
-        <v>0.726</v>
+        <v>0.76</v>
       </c>
       <c r="F38" t="n" s="3">
-        <v>0.662</v>
+        <v>0.752</v>
       </c>
       <c r="G38" t="n" s="3">
-        <v>0.679</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C39" t="n" s="3">
-        <v>0.692</v>
+        <v>0.763</v>
       </c>
       <c r="D39" t="n" s="3">
-        <v>0.63</v>
+        <v>0.753</v>
       </c>
       <c r="E39" t="n" s="3">
-        <v>0.619</v>
+        <v>0.709</v>
       </c>
       <c r="F39" t="n" s="3">
-        <v>0.603</v>
+        <v>0.723</v>
       </c>
       <c r="G39" t="n" s="3">
-        <v>0.692</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C40" t="n" s="3">
-        <v>0.695</v>
+        <v>0.688</v>
       </c>
       <c r="D40" t="n" s="3">
-        <v>0.677</v>
+        <v>0.6</v>
       </c>
       <c r="E40" t="n" s="3">
-        <v>0.626</v>
+        <v>0.669</v>
       </c>
       <c r="F40" t="n" s="3">
-        <v>0.625</v>
+        <v>0.622</v>
       </c>
       <c r="G40" t="n" s="3">
-        <v>0.695</v>
+        <v>0.688</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C41" t="n" s="3">
-        <v>0.766</v>
+        <v>0.75</v>
       </c>
       <c r="D41" t="n" s="3">
-        <v>0.698</v>
+        <v>0.711</v>
       </c>
       <c r="E41" t="n" s="3">
-        <v>0.803</v>
+        <v>0.748</v>
       </c>
       <c r="F41" t="n" s="3">
-        <v>0.737</v>
+        <v>0.728</v>
       </c>
       <c r="G41" t="n" s="3">
-        <v>0.766</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C42" t="n" s="3">
         <v>0.763</v>
       </c>
       <c r="D42" t="n" s="3">
-        <v>0.697</v>
+        <v>0.725</v>
       </c>
       <c r="E42" t="n" s="3">
-        <v>0.771</v>
+        <v>0.701</v>
       </c>
       <c r="F42" t="n" s="3">
-        <v>0.727</v>
+        <v>0.707</v>
       </c>
       <c r="G42" t="n" s="3">
         <v>0.763</v>
@@ -1194,392 +1218,576 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C43" t="n" s="3">
-        <v>0.724</v>
+        <v>0.747</v>
       </c>
       <c r="D43" t="n" s="3">
-        <v>0.646</v>
+        <v>0.674</v>
       </c>
       <c r="E43" t="n" s="3">
-        <v>0.78</v>
+        <v>0.739</v>
       </c>
       <c r="F43" t="n" s="3">
-        <v>0.684</v>
+        <v>0.701</v>
       </c>
       <c r="G43" t="n" s="3">
-        <v>0.724</v>
+        <v>0.747</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C44" t="n" s="3">
-        <v>0.724</v>
+        <v>0.708</v>
       </c>
       <c r="D44" t="n" s="3">
-        <v>0.639</v>
+        <v>0.618</v>
       </c>
       <c r="E44" t="n" s="3">
-        <v>0.772</v>
+        <v>0.738</v>
       </c>
       <c r="F44" t="n" s="3">
-        <v>0.677</v>
+        <v>0.651</v>
       </c>
       <c r="G44" t="n" s="3">
-        <v>0.724</v>
+        <v>0.708</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C45" t="n" s="3">
-        <v>0.789</v>
+        <v>0.662</v>
       </c>
       <c r="D45" t="n" s="3">
-        <v>0.738</v>
+        <v>0.638</v>
       </c>
       <c r="E45" t="n" s="3">
-        <v>0.753</v>
+        <v>0.741</v>
       </c>
       <c r="F45" t="n" s="3">
-        <v>0.744</v>
+        <v>0.652</v>
       </c>
       <c r="G45" t="n" s="3">
-        <v>0.789</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="C46" t="n" s="3">
-        <v>0.773</v>
+        <v>0.679</v>
       </c>
       <c r="D46" t="n" s="3">
-        <v>0.77</v>
+        <v>0.657</v>
       </c>
       <c r="E46" t="n" s="3">
-        <v>0.76</v>
+        <v>0.726</v>
       </c>
       <c r="F46" t="n" s="3">
-        <v>0.755</v>
+        <v>0.662</v>
       </c>
       <c r="G46" t="n" s="3">
-        <v>0.773</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="C47" t="n" s="3">
-        <v>0.812</v>
+        <v>0.692</v>
       </c>
       <c r="D47" t="n" s="3">
-        <v>0.798</v>
+        <v>0.63</v>
       </c>
       <c r="E47" t="n" s="3">
-        <v>0.79</v>
+        <v>0.619</v>
       </c>
       <c r="F47" t="n" s="3">
-        <v>0.789</v>
+        <v>0.603</v>
       </c>
       <c r="G47" t="n" s="3">
-        <v>0.812</v>
+        <v>0.692</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C48" t="n" s="3">
-        <v>0.675</v>
+        <v>0.695</v>
       </c>
       <c r="D48" t="n" s="3">
-        <v>0.603</v>
+        <v>0.677</v>
       </c>
       <c r="E48" t="n" s="3">
-        <v>0.755</v>
+        <v>0.626</v>
       </c>
       <c r="F48" t="n" s="3">
         <v>0.625</v>
       </c>
       <c r="G48" t="n" s="3">
-        <v>0.675</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C49" t="n" s="3">
-        <v>0.74</v>
+        <v>0.766</v>
       </c>
       <c r="D49" t="n" s="3">
-        <v>0.807</v>
+        <v>0.698</v>
       </c>
       <c r="E49" t="n" s="3">
-        <v>0.744</v>
+        <v>0.803</v>
       </c>
       <c r="F49" t="n" s="3">
-        <v>0.743</v>
+        <v>0.737</v>
       </c>
       <c r="G49" t="n" s="3">
-        <v>0.74</v>
+        <v>0.766</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="C50" t="n" s="3">
-        <v>0.782</v>
+        <v>0.763</v>
       </c>
       <c r="D50" t="n" s="3">
-        <v>0.734</v>
+        <v>0.697</v>
       </c>
       <c r="E50" t="n" s="3">
-        <v>0.83</v>
+        <v>0.771</v>
       </c>
       <c r="F50" t="n" s="3">
-        <v>0.764</v>
+        <v>0.727</v>
       </c>
       <c r="G50" t="n" s="3">
-        <v>0.782</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C51" t="n" s="3">
-        <v>0.795</v>
+        <v>0.724</v>
       </c>
       <c r="D51" t="n" s="3">
-        <v>0.736</v>
+        <v>0.646</v>
       </c>
       <c r="E51" t="n" s="3">
-        <v>0.854</v>
+        <v>0.78</v>
       </c>
       <c r="F51" t="n" s="3">
-        <v>0.777</v>
+        <v>0.684</v>
       </c>
       <c r="G51" t="n" s="3">
-        <v>0.795</v>
+        <v>0.724</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C52" t="n" s="3">
-        <v>0.825</v>
+        <v>0.724</v>
       </c>
       <c r="D52" t="n" s="3">
-        <v>0.808</v>
+        <v>0.639</v>
       </c>
       <c r="E52" t="n" s="3">
-        <v>0.796</v>
+        <v>0.772</v>
       </c>
       <c r="F52" t="n" s="3">
-        <v>0.799</v>
+        <v>0.677</v>
       </c>
       <c r="G52" t="n" s="3">
-        <v>0.825</v>
+        <v>0.724</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="C53" t="n" s="3">
-        <v>0.808</v>
+        <v>0.789</v>
       </c>
       <c r="D53" t="n" s="3">
-        <v>0.772</v>
+        <v>0.738</v>
       </c>
       <c r="E53" t="n" s="3">
-        <v>0.781</v>
+        <v>0.753</v>
       </c>
       <c r="F53" t="n" s="3">
-        <v>0.772</v>
+        <v>0.744</v>
       </c>
       <c r="G53" t="n" s="3">
-        <v>0.808</v>
+        <v>0.789</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C54" t="n" s="3">
-        <v>0.802</v>
+        <v>0.773</v>
       </c>
       <c r="D54" t="n" s="3">
-        <v>0.754</v>
+        <v>0.77</v>
       </c>
       <c r="E54" t="n" s="3">
-        <v>0.787</v>
+        <v>0.76</v>
       </c>
       <c r="F54" t="n" s="3">
-        <v>0.769</v>
+        <v>0.755</v>
       </c>
       <c r="G54" t="n" s="3">
-        <v>0.802</v>
+        <v>0.773</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C55" t="n" s="3">
-        <v>0.662</v>
+        <v>0.812</v>
       </c>
       <c r="D55" t="n" s="3">
-        <v>0.589</v>
+        <v>0.798</v>
       </c>
       <c r="E55" t="n" s="3">
-        <v>0.738</v>
+        <v>0.79</v>
       </c>
       <c r="F55" t="n" s="3">
-        <v>0.613</v>
+        <v>0.789</v>
       </c>
       <c r="G55" t="n" s="3">
-        <v>0.662</v>
+        <v>0.812</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C56" t="n" s="3">
-        <v>0.782</v>
+        <v>0.675</v>
       </c>
       <c r="D56" t="n" s="3">
-        <v>0.718</v>
+        <v>0.603</v>
       </c>
       <c r="E56" t="n" s="3">
-        <v>0.778</v>
+        <v>0.755</v>
       </c>
       <c r="F56" t="n" s="3">
-        <v>0.741</v>
+        <v>0.625</v>
       </c>
       <c r="G56" t="n" s="3">
-        <v>0.782</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="C57" t="n" s="3">
-        <v>0.808</v>
+        <v>0.74</v>
       </c>
       <c r="D57" t="n" s="3">
-        <v>0.783</v>
+        <v>0.807</v>
       </c>
       <c r="E57" t="n" s="3">
-        <v>0.77</v>
+        <v>0.744</v>
       </c>
       <c r="F57" t="n" s="3">
-        <v>0.776</v>
+        <v>0.743</v>
       </c>
       <c r="G57" t="n" s="3">
-        <v>0.808</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="C58" t="n" s="3">
-        <v>0.708</v>
+        <v>0.782</v>
       </c>
       <c r="D58" t="n" s="3">
-        <v>0.637</v>
+        <v>0.734</v>
       </c>
       <c r="E58" t="n" s="3">
-        <v>0.79</v>
+        <v>0.83</v>
       </c>
       <c r="F58" t="n" s="3">
-        <v>0.674</v>
+        <v>0.764</v>
       </c>
       <c r="G58" t="n" s="3">
-        <v>0.708</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="C59" t="n" s="3">
+        <v>0.795</v>
+      </c>
+      <c r="D59" t="n" s="3">
+        <v>0.736</v>
+      </c>
+      <c r="E59" t="n" s="3">
+        <v>0.854</v>
+      </c>
+      <c r="F59" t="n" s="3">
+        <v>0.777</v>
+      </c>
+      <c r="G59" t="n" s="3">
+        <v>0.795</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="C60" t="n" s="3">
+        <v>0.825</v>
+      </c>
+      <c r="D60" t="n" s="3">
+        <v>0.808</v>
+      </c>
+      <c r="E60" t="n" s="3">
+        <v>0.796</v>
+      </c>
+      <c r="F60" t="n" s="3">
+        <v>0.799</v>
+      </c>
+      <c r="G60" t="n" s="3">
+        <v>0.825</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B61" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="B59" t="s" s="2">
-        <v>15</v>
-      </c>
-      <c r="C59" t="n" s="3">
+      <c r="C61" t="n" s="3">
+        <v>0.808</v>
+      </c>
+      <c r="D61" t="n" s="3">
+        <v>0.772</v>
+      </c>
+      <c r="E61" t="n" s="3">
+        <v>0.781</v>
+      </c>
+      <c r="F61" t="n" s="3">
+        <v>0.772</v>
+      </c>
+      <c r="G61" t="n" s="3">
+        <v>0.808</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="C62" t="n" s="3">
+        <v>0.802</v>
+      </c>
+      <c r="D62" t="n" s="3">
+        <v>0.754</v>
+      </c>
+      <c r="E62" t="n" s="3">
+        <v>0.787</v>
+      </c>
+      <c r="F62" t="n" s="3">
+        <v>0.769</v>
+      </c>
+      <c r="G62" t="n" s="3">
+        <v>0.802</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B63" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C63" t="n" s="3">
+        <v>0.662</v>
+      </c>
+      <c r="D63" t="n" s="3">
+        <v>0.589</v>
+      </c>
+      <c r="E63" t="n" s="3">
+        <v>0.738</v>
+      </c>
+      <c r="F63" t="n" s="3">
+        <v>0.613</v>
+      </c>
+      <c r="G63" t="n" s="3">
+        <v>0.662</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B64" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="C64" t="n" s="3">
+        <v>0.782</v>
+      </c>
+      <c r="D64" t="n" s="3">
+        <v>0.718</v>
+      </c>
+      <c r="E64" t="n" s="3">
+        <v>0.778</v>
+      </c>
+      <c r="F64" t="n" s="3">
+        <v>0.741</v>
+      </c>
+      <c r="G64" t="n" s="3">
+        <v>0.782</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="C65" t="n" s="3">
+        <v>0.808</v>
+      </c>
+      <c r="D65" t="n" s="3">
+        <v>0.783</v>
+      </c>
+      <c r="E65" t="n" s="3">
+        <v>0.77</v>
+      </c>
+      <c r="F65" t="n" s="3">
+        <v>0.776</v>
+      </c>
+      <c r="G65" t="n" s="3">
+        <v>0.808</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B66" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="C66" t="n" s="3">
+        <v>0.708</v>
+      </c>
+      <c r="D66" t="n" s="3">
+        <v>0.637</v>
+      </c>
+      <c r="E66" t="n" s="3">
+        <v>0.79</v>
+      </c>
+      <c r="F66" t="n" s="3">
+        <v>0.674</v>
+      </c>
+      <c r="G66" t="n" s="3">
+        <v>0.708</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B67" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="C67" t="n" s="3">
         <v>0.679</v>
       </c>
-      <c r="D59" t="n" s="3">
+      <c r="D67" t="n" s="3">
         <v>0.602</v>
       </c>
-      <c r="E59" t="n" s="3">
+      <c r="E67" t="n" s="3">
         <v>0.747</v>
       </c>
-      <c r="F59" t="n" s="3">
+      <c r="F67" t="n" s="3">
         <v>0.624</v>
       </c>
-      <c r="G59" t="n" s="3">
+      <c r="G67" t="n" s="3">
         <v>0.679</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Export the newest results with cleaned data & custom taxonomy
</commit_message>
<xml_diff>
--- a/clarity-pipeline/src/test/resources/evaluation/12_14_2025.xlsx
+++ b/clarity-pipeline/src/test/resources/evaluation/12_14_2025.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="50">
   <si>
     <t>Name</t>
   </si>
@@ -101,30 +101,30 @@
     <t>Llama 3.3 70B</t>
   </si>
   <si>
+    <t>extended-evasion-based:best-guess:few-shot:v2</t>
+  </si>
+  <si>
+    <t>extended-evasion-based:best-guess:few-shot:v1</t>
+  </si>
+  <si>
+    <t>extended-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>rag:evasion-based:single:few-shot:v4</t>
+  </si>
+  <si>
+    <t>rag:evasion-based:single:few-shot:v3</t>
+  </si>
+  <si>
+    <t>rag:evasion-based:single:few-shot:v2</t>
+  </si>
+  <si>
+    <t>rag:evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
     <t>pag:evasion-based:few-shot:v1</t>
   </si>
   <si>
-    <t>extended-evasion-based:best-guess:few-shot:v2</t>
-  </si>
-  <si>
-    <t>extended-evasion-based:best-guess:few-shot:v1</t>
-  </si>
-  <si>
-    <t>extended-evasion-based:single:few-shot:v1</t>
-  </si>
-  <si>
-    <t>rag:evasion-based:single:few-shot:v4</t>
-  </si>
-  <si>
-    <t>rag:evasion-based:single:few-shot:v3</t>
-  </si>
-  <si>
-    <t>rag:evasion-based:single:few-shot:v2</t>
-  </si>
-  <si>
-    <t>rag:evasion-based:single:few-shot:v1</t>
-  </si>
-  <si>
     <t>GPT-OSS-120B</t>
   </si>
   <si>
@@ -146,6 +146,15 @@
     <t>GPT 5.1</t>
   </si>
   <si>
+    <t>cleaned:custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>custom-evasion-based:single:few-shot:v1</t>
+  </si>
+  <si>
+    <t>rag:evasion-based:judgement:few-shot:v1</t>
+  </si>
+  <si>
     <t>rag:evasion-based:single:few-shot:v5</t>
   </si>
   <si>
@@ -153,9 +162,6 @@
   </si>
   <si>
     <t>pag:few-shot:v1</t>
-  </si>
-  <si>
-    <t>rag:evasion-based:judgement:few-shot:v1</t>
   </si>
 </sst>
 </file>
@@ -238,7 +244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="14.95703125" customWidth="true" bestFit="true"/>
@@ -787,19 +793,19 @@
         <v>29</v>
       </c>
       <c r="C24" t="n" s="3">
-        <v>0.753</v>
+        <v>0.685</v>
       </c>
       <c r="D24" t="n" s="3">
-        <v>0.856</v>
+        <v>0.664</v>
       </c>
       <c r="E24" t="n" s="3">
-        <v>0.595</v>
+        <v>0.575</v>
       </c>
       <c r="F24" t="n" s="3">
-        <v>0.636</v>
+        <v>0.588</v>
       </c>
       <c r="G24" t="n" s="3">
-        <v>0.753</v>
+        <v>0.685</v>
       </c>
     </row>
     <row r="25">
@@ -810,19 +816,19 @@
         <v>30</v>
       </c>
       <c r="C25" t="n" s="3">
-        <v>0.685</v>
+        <v>0.76</v>
       </c>
       <c r="D25" t="n" s="3">
-        <v>0.664</v>
+        <v>0.784</v>
       </c>
       <c r="E25" t="n" s="3">
-        <v>0.575</v>
+        <v>0.542</v>
       </c>
       <c r="F25" t="n" s="3">
-        <v>0.588</v>
+        <v>0.593</v>
       </c>
       <c r="G25" t="n" s="3">
-        <v>0.685</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="26">
@@ -833,19 +839,19 @@
         <v>31</v>
       </c>
       <c r="C26" t="n" s="3">
-        <v>0.76</v>
+        <v>0.747</v>
       </c>
       <c r="D26" t="n" s="3">
-        <v>0.784</v>
+        <v>0.72</v>
       </c>
       <c r="E26" t="n" s="3">
-        <v>0.542</v>
+        <v>0.595</v>
       </c>
       <c r="F26" t="n" s="3">
-        <v>0.593</v>
+        <v>0.636</v>
       </c>
       <c r="G26" t="n" s="3">
-        <v>0.76</v>
+        <v>0.747</v>
       </c>
     </row>
     <row r="27">
@@ -856,19 +862,19 @@
         <v>32</v>
       </c>
       <c r="C27" t="n" s="3">
-        <v>0.747</v>
+        <v>0.782</v>
       </c>
       <c r="D27" t="n" s="3">
-        <v>0.72</v>
+        <v>0.804</v>
       </c>
       <c r="E27" t="n" s="3">
-        <v>0.595</v>
+        <v>0.664</v>
       </c>
       <c r="F27" t="n" s="3">
-        <v>0.636</v>
+        <v>0.692</v>
       </c>
       <c r="G27" t="n" s="3">
-        <v>0.747</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="28">
@@ -879,19 +885,19 @@
         <v>33</v>
       </c>
       <c r="C28" t="n" s="3">
-        <v>0.782</v>
+        <v>0.731</v>
       </c>
       <c r="D28" t="n" s="3">
-        <v>0.804</v>
+        <v>0.756</v>
       </c>
       <c r="E28" t="n" s="3">
-        <v>0.664</v>
+        <v>0.558</v>
       </c>
       <c r="F28" t="n" s="3">
-        <v>0.692</v>
+        <v>0.591</v>
       </c>
       <c r="G28" t="n" s="3">
-        <v>0.782</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="29">
@@ -902,19 +908,19 @@
         <v>34</v>
       </c>
       <c r="C29" t="n" s="3">
-        <v>0.731</v>
+        <v>0.769</v>
       </c>
       <c r="D29" t="n" s="3">
-        <v>0.756</v>
+        <v>0.783</v>
       </c>
       <c r="E29" t="n" s="3">
-        <v>0.558</v>
+        <v>0.629</v>
       </c>
       <c r="F29" t="n" s="3">
-        <v>0.591</v>
+        <v>0.663</v>
       </c>
       <c r="G29" t="n" s="3">
-        <v>0.731</v>
+        <v>0.769</v>
       </c>
     </row>
     <row r="30">
@@ -925,19 +931,19 @@
         <v>35</v>
       </c>
       <c r="C30" t="n" s="3">
-        <v>0.769</v>
+        <v>0.737</v>
       </c>
       <c r="D30" t="n" s="3">
-        <v>0.783</v>
+        <v>0.772</v>
       </c>
       <c r="E30" t="n" s="3">
-        <v>0.629</v>
+        <v>0.563</v>
       </c>
       <c r="F30" t="n" s="3">
-        <v>0.663</v>
+        <v>0.599</v>
       </c>
       <c r="G30" t="n" s="3">
-        <v>0.769</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="31">
@@ -945,22 +951,22 @@
         <v>28</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C31" t="n" s="3">
-        <v>0.737</v>
+        <v>0.731</v>
       </c>
       <c r="D31" t="n" s="3">
-        <v>0.772</v>
+        <v>0.673</v>
       </c>
       <c r="E31" t="n" s="3">
-        <v>0.563</v>
+        <v>0.599</v>
       </c>
       <c r="F31" t="n" s="3">
-        <v>0.599</v>
+        <v>0.601</v>
       </c>
       <c r="G31" t="n" s="3">
-        <v>0.737</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="32">
@@ -968,22 +974,22 @@
         <v>28</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C32" t="n" s="3">
-        <v>0.731</v>
+        <v>0.753</v>
       </c>
       <c r="D32" t="n" s="3">
-        <v>0.673</v>
+        <v>0.867</v>
       </c>
       <c r="E32" t="n" s="3">
-        <v>0.599</v>
+        <v>0.602</v>
       </c>
       <c r="F32" t="n" s="3">
-        <v>0.601</v>
+        <v>0.636</v>
       </c>
       <c r="G32" t="n" s="3">
-        <v>0.731</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="33">
@@ -991,22 +997,22 @@
         <v>28</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C33" t="n" s="3">
-        <v>0.753</v>
+        <v>0.695</v>
       </c>
       <c r="D33" t="n" s="3">
-        <v>0.867</v>
+        <v>0.637</v>
       </c>
       <c r="E33" t="n" s="3">
         <v>0.602</v>
       </c>
       <c r="F33" t="n" s="3">
-        <v>0.636</v>
+        <v>0.553</v>
       </c>
       <c r="G33" t="n" s="3">
-        <v>0.753</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="34">
@@ -1014,22 +1020,22 @@
         <v>28</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C34" t="n" s="3">
-        <v>0.695</v>
+        <v>0.753</v>
       </c>
       <c r="D34" t="n" s="3">
-        <v>0.637</v>
+        <v>0.856</v>
       </c>
       <c r="E34" t="n" s="3">
-        <v>0.602</v>
+        <v>0.595</v>
       </c>
       <c r="F34" t="n" s="3">
-        <v>0.553</v>
+        <v>0.636</v>
       </c>
       <c r="G34" t="n" s="3">
-        <v>0.695</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="35">
@@ -1037,22 +1043,22 @@
         <v>37</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C35" t="n" s="3">
+        <v>0.744</v>
+      </c>
+      <c r="D35" t="n" s="3">
+        <v>0.728</v>
+      </c>
+      <c r="E35" t="n" s="3">
+        <v>0.707</v>
+      </c>
+      <c r="F35" t="n" s="3">
         <v>0.708</v>
       </c>
-      <c r="D35" t="n" s="3">
-        <v>0.682</v>
-      </c>
-      <c r="E35" t="n" s="3">
-        <v>0.655</v>
-      </c>
-      <c r="F35" t="n" s="3">
-        <v>0.663</v>
-      </c>
       <c r="G35" t="n" s="3">
-        <v>0.708</v>
+        <v>0.744</v>
       </c>
     </row>
     <row r="36">
@@ -1063,19 +1069,19 @@
         <v>34</v>
       </c>
       <c r="C36" t="n" s="3">
-        <v>0.744</v>
+        <v>0.772</v>
       </c>
       <c r="D36" t="n" s="3">
-        <v>0.728</v>
+        <v>0.755</v>
       </c>
       <c r="E36" t="n" s="3">
-        <v>0.707</v>
+        <v>0.759</v>
       </c>
       <c r="F36" t="n" s="3">
-        <v>0.708</v>
+        <v>0.752</v>
       </c>
       <c r="G36" t="n" s="3">
-        <v>0.744</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="37">
@@ -1083,22 +1089,22 @@
         <v>37</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C37" t="n" s="3">
-        <v>0.772</v>
+        <v>0.782</v>
       </c>
       <c r="D37" t="n" s="3">
-        <v>0.755</v>
+        <v>0.745</v>
       </c>
       <c r="E37" t="n" s="3">
-        <v>0.759</v>
+        <v>0.76</v>
       </c>
       <c r="F37" t="n" s="3">
         <v>0.752</v>
       </c>
       <c r="G37" t="n" s="3">
-        <v>0.772</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="38">
@@ -1106,22 +1112,22 @@
         <v>37</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C38" t="n" s="3">
-        <v>0.782</v>
+        <v>0.763</v>
       </c>
       <c r="D38" t="n" s="3">
-        <v>0.745</v>
+        <v>0.753</v>
       </c>
       <c r="E38" t="n" s="3">
-        <v>0.76</v>
+        <v>0.709</v>
       </c>
       <c r="F38" t="n" s="3">
-        <v>0.752</v>
+        <v>0.723</v>
       </c>
       <c r="G38" t="n" s="3">
-        <v>0.782</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="39">
@@ -1129,22 +1135,22 @@
         <v>37</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C39" t="n" s="3">
-        <v>0.763</v>
+        <v>0.688</v>
       </c>
       <c r="D39" t="n" s="3">
-        <v>0.753</v>
+        <v>0.6</v>
       </c>
       <c r="E39" t="n" s="3">
-        <v>0.709</v>
+        <v>0.669</v>
       </c>
       <c r="F39" t="n" s="3">
-        <v>0.723</v>
+        <v>0.622</v>
       </c>
       <c r="G39" t="n" s="3">
-        <v>0.763</v>
+        <v>0.688</v>
       </c>
     </row>
     <row r="40">
@@ -1152,22 +1158,22 @@
         <v>37</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C40" t="n" s="3">
-        <v>0.688</v>
+        <v>0.75</v>
       </c>
       <c r="D40" t="n" s="3">
-        <v>0.6</v>
+        <v>0.711</v>
       </c>
       <c r="E40" t="n" s="3">
-        <v>0.669</v>
+        <v>0.748</v>
       </c>
       <c r="F40" t="n" s="3">
-        <v>0.622</v>
+        <v>0.728</v>
       </c>
       <c r="G40" t="n" s="3">
-        <v>0.688</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="41">
@@ -1175,22 +1181,22 @@
         <v>37</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="C41" t="n" s="3">
-        <v>0.75</v>
+        <v>0.763</v>
       </c>
       <c r="D41" t="n" s="3">
-        <v>0.711</v>
+        <v>0.725</v>
       </c>
       <c r="E41" t="n" s="3">
-        <v>0.748</v>
+        <v>0.701</v>
       </c>
       <c r="F41" t="n" s="3">
-        <v>0.728</v>
+        <v>0.707</v>
       </c>
       <c r="G41" t="n" s="3">
-        <v>0.75</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="42">
@@ -1198,22 +1204,22 @@
         <v>37</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C42" t="n" s="3">
-        <v>0.763</v>
+        <v>0.747</v>
       </c>
       <c r="D42" t="n" s="3">
-        <v>0.725</v>
+        <v>0.674</v>
       </c>
       <c r="E42" t="n" s="3">
+        <v>0.739</v>
+      </c>
+      <c r="F42" t="n" s="3">
         <v>0.701</v>
       </c>
-      <c r="F42" t="n" s="3">
-        <v>0.707</v>
-      </c>
       <c r="G42" t="n" s="3">
-        <v>0.763</v>
+        <v>0.747</v>
       </c>
     </row>
     <row r="43">
@@ -1221,22 +1227,22 @@
         <v>37</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C43" t="n" s="3">
-        <v>0.747</v>
+        <v>0.708</v>
       </c>
       <c r="D43" t="n" s="3">
-        <v>0.674</v>
+        <v>0.618</v>
       </c>
       <c r="E43" t="n" s="3">
-        <v>0.739</v>
+        <v>0.738</v>
       </c>
       <c r="F43" t="n" s="3">
-        <v>0.701</v>
+        <v>0.651</v>
       </c>
       <c r="G43" t="n" s="3">
-        <v>0.747</v>
+        <v>0.708</v>
       </c>
     </row>
     <row r="44">
@@ -1244,19 +1250,19 @@
         <v>37</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C44" t="n" s="3">
         <v>0.708</v>
       </c>
       <c r="D44" t="n" s="3">
-        <v>0.618</v>
+        <v>0.682</v>
       </c>
       <c r="E44" t="n" s="3">
-        <v>0.738</v>
+        <v>0.655</v>
       </c>
       <c r="F44" t="n" s="3">
-        <v>0.651</v>
+        <v>0.663</v>
       </c>
       <c r="G44" t="n" s="3">
         <v>0.708</v>
@@ -1267,22 +1273,22 @@
         <v>41</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C45" t="n" s="3">
+        <v>0.679</v>
+      </c>
+      <c r="D45" t="n" s="3">
+        <v>0.657</v>
+      </c>
+      <c r="E45" t="n" s="3">
+        <v>0.726</v>
+      </c>
+      <c r="F45" t="n" s="3">
         <v>0.662</v>
       </c>
-      <c r="D45" t="n" s="3">
-        <v>0.638</v>
-      </c>
-      <c r="E45" t="n" s="3">
-        <v>0.741</v>
-      </c>
-      <c r="F45" t="n" s="3">
-        <v>0.652</v>
-      </c>
       <c r="G45" t="n" s="3">
-        <v>0.662</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="46">
@@ -1290,22 +1296,22 @@
         <v>41</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C46" t="n" s="3">
-        <v>0.679</v>
+        <v>0.692</v>
       </c>
       <c r="D46" t="n" s="3">
-        <v>0.657</v>
+        <v>0.63</v>
       </c>
       <c r="E46" t="n" s="3">
-        <v>0.726</v>
+        <v>0.619</v>
       </c>
       <c r="F46" t="n" s="3">
-        <v>0.662</v>
+        <v>0.603</v>
       </c>
       <c r="G46" t="n" s="3">
-        <v>0.679</v>
+        <v>0.692</v>
       </c>
     </row>
     <row r="47">
@@ -1313,22 +1319,22 @@
         <v>41</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C47" t="n" s="3">
-        <v>0.692</v>
+        <v>0.695</v>
       </c>
       <c r="D47" t="n" s="3">
-        <v>0.63</v>
+        <v>0.677</v>
       </c>
       <c r="E47" t="n" s="3">
-        <v>0.619</v>
+        <v>0.626</v>
       </c>
       <c r="F47" t="n" s="3">
-        <v>0.603</v>
+        <v>0.625</v>
       </c>
       <c r="G47" t="n" s="3">
-        <v>0.692</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="48">
@@ -1336,22 +1342,22 @@
         <v>41</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C48" t="n" s="3">
-        <v>0.695</v>
+        <v>0.662</v>
       </c>
       <c r="D48" t="n" s="3">
-        <v>0.677</v>
+        <v>0.638</v>
       </c>
       <c r="E48" t="n" s="3">
-        <v>0.626</v>
+        <v>0.741</v>
       </c>
       <c r="F48" t="n" s="3">
-        <v>0.625</v>
+        <v>0.652</v>
       </c>
       <c r="G48" t="n" s="3">
-        <v>0.695</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="49">
@@ -1454,19 +1460,19 @@
         <v>44</v>
       </c>
       <c r="C53" t="n" s="3">
-        <v>0.789</v>
+        <v>0.804</v>
       </c>
       <c r="D53" t="n" s="3">
-        <v>0.738</v>
+        <v>0.801</v>
       </c>
       <c r="E53" t="n" s="3">
-        <v>0.753</v>
+        <v>0.729</v>
       </c>
       <c r="F53" t="n" s="3">
-        <v>0.744</v>
+        <v>0.757</v>
       </c>
       <c r="G53" t="n" s="3">
-        <v>0.789</v>
+        <v>0.804</v>
       </c>
     </row>
     <row r="54">
@@ -1477,19 +1483,19 @@
         <v>45</v>
       </c>
       <c r="C54" t="n" s="3">
-        <v>0.773</v>
+        <v>0.812</v>
       </c>
       <c r="D54" t="n" s="3">
-        <v>0.77</v>
+        <v>0.808</v>
       </c>
       <c r="E54" t="n" s="3">
-        <v>0.76</v>
+        <v>0.767</v>
       </c>
       <c r="F54" t="n" s="3">
-        <v>0.755</v>
+        <v>0.778</v>
       </c>
       <c r="G54" t="n" s="3">
-        <v>0.773</v>
+        <v>0.812</v>
       </c>
     </row>
     <row r="55">
@@ -1497,22 +1503,22 @@
         <v>43</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C55" t="n" s="3">
-        <v>0.812</v>
+        <v>0.74</v>
       </c>
       <c r="D55" t="n" s="3">
-        <v>0.798</v>
+        <v>0.807</v>
       </c>
       <c r="E55" t="n" s="3">
-        <v>0.79</v>
+        <v>0.744</v>
       </c>
       <c r="F55" t="n" s="3">
-        <v>0.789</v>
+        <v>0.743</v>
       </c>
       <c r="G55" t="n" s="3">
-        <v>0.812</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="56">
@@ -1523,19 +1529,19 @@
         <v>46</v>
       </c>
       <c r="C56" t="n" s="3">
-        <v>0.675</v>
+        <v>0.782</v>
       </c>
       <c r="D56" t="n" s="3">
-        <v>0.603</v>
+        <v>0.734</v>
       </c>
       <c r="E56" t="n" s="3">
-        <v>0.755</v>
+        <v>0.83</v>
       </c>
       <c r="F56" t="n" s="3">
-        <v>0.625</v>
+        <v>0.764</v>
       </c>
       <c r="G56" t="n" s="3">
-        <v>0.675</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="57">
@@ -1543,22 +1549,22 @@
         <v>43</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C57" t="n" s="3">
-        <v>0.74</v>
+        <v>0.795</v>
       </c>
       <c r="D57" t="n" s="3">
-        <v>0.807</v>
+        <v>0.736</v>
       </c>
       <c r="E57" t="n" s="3">
-        <v>0.744</v>
+        <v>0.854</v>
       </c>
       <c r="F57" t="n" s="3">
-        <v>0.743</v>
+        <v>0.777</v>
       </c>
       <c r="G57" t="n" s="3">
-        <v>0.74</v>
+        <v>0.795</v>
       </c>
     </row>
     <row r="58">
@@ -1566,22 +1572,22 @@
         <v>43</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C58" t="n" s="3">
-        <v>0.782</v>
+        <v>0.825</v>
       </c>
       <c r="D58" t="n" s="3">
-        <v>0.734</v>
+        <v>0.808</v>
       </c>
       <c r="E58" t="n" s="3">
-        <v>0.83</v>
+        <v>0.796</v>
       </c>
       <c r="F58" t="n" s="3">
-        <v>0.764</v>
+        <v>0.799</v>
       </c>
       <c r="G58" t="n" s="3">
-        <v>0.782</v>
+        <v>0.825</v>
       </c>
     </row>
     <row r="59">
@@ -1589,22 +1595,22 @@
         <v>43</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C59" t="n" s="3">
-        <v>0.795</v>
+        <v>0.808</v>
       </c>
       <c r="D59" t="n" s="3">
-        <v>0.736</v>
+        <v>0.772</v>
       </c>
       <c r="E59" t="n" s="3">
-        <v>0.854</v>
+        <v>0.781</v>
       </c>
       <c r="F59" t="n" s="3">
-        <v>0.777</v>
+        <v>0.772</v>
       </c>
       <c r="G59" t="n" s="3">
-        <v>0.795</v>
+        <v>0.808</v>
       </c>
     </row>
     <row r="60">
@@ -1612,22 +1618,22 @@
         <v>43</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C60" t="n" s="3">
-        <v>0.825</v>
+        <v>0.802</v>
       </c>
       <c r="D60" t="n" s="3">
-        <v>0.808</v>
+        <v>0.754</v>
       </c>
       <c r="E60" t="n" s="3">
-        <v>0.796</v>
+        <v>0.787</v>
       </c>
       <c r="F60" t="n" s="3">
-        <v>0.799</v>
+        <v>0.769</v>
       </c>
       <c r="G60" t="n" s="3">
-        <v>0.825</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="61">
@@ -1635,22 +1641,22 @@
         <v>43</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C61" t="n" s="3">
-        <v>0.808</v>
+        <v>0.662</v>
       </c>
       <c r="D61" t="n" s="3">
-        <v>0.772</v>
+        <v>0.589</v>
       </c>
       <c r="E61" t="n" s="3">
-        <v>0.781</v>
+        <v>0.738</v>
       </c>
       <c r="F61" t="n" s="3">
-        <v>0.772</v>
+        <v>0.613</v>
       </c>
       <c r="G61" t="n" s="3">
-        <v>0.808</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="62">
@@ -1658,22 +1664,22 @@
         <v>43</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C62" t="n" s="3">
-        <v>0.802</v>
+        <v>0.782</v>
       </c>
       <c r="D62" t="n" s="3">
-        <v>0.754</v>
+        <v>0.718</v>
       </c>
       <c r="E62" t="n" s="3">
-        <v>0.787</v>
+        <v>0.778</v>
       </c>
       <c r="F62" t="n" s="3">
-        <v>0.769</v>
+        <v>0.741</v>
       </c>
       <c r="G62" t="n" s="3">
-        <v>0.802</v>
+        <v>0.782</v>
       </c>
     </row>
     <row r="63">
@@ -1681,22 +1687,22 @@
         <v>43</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C63" t="n" s="3">
-        <v>0.662</v>
+        <v>0.808</v>
       </c>
       <c r="D63" t="n" s="3">
-        <v>0.589</v>
+        <v>0.783</v>
       </c>
       <c r="E63" t="n" s="3">
-        <v>0.738</v>
+        <v>0.77</v>
       </c>
       <c r="F63" t="n" s="3">
-        <v>0.613</v>
+        <v>0.776</v>
       </c>
       <c r="G63" t="n" s="3">
-        <v>0.662</v>
+        <v>0.808</v>
       </c>
     </row>
     <row r="64">
@@ -1704,22 +1710,22 @@
         <v>43</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C64" t="n" s="3">
-        <v>0.782</v>
+        <v>0.708</v>
       </c>
       <c r="D64" t="n" s="3">
-        <v>0.718</v>
+        <v>0.637</v>
       </c>
       <c r="E64" t="n" s="3">
-        <v>0.778</v>
+        <v>0.79</v>
       </c>
       <c r="F64" t="n" s="3">
-        <v>0.741</v>
+        <v>0.674</v>
       </c>
       <c r="G64" t="n" s="3">
-        <v>0.782</v>
+        <v>0.708</v>
       </c>
     </row>
     <row r="65">
@@ -1727,22 +1733,22 @@
         <v>43</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C65" t="n" s="3">
-        <v>0.808</v>
+        <v>0.679</v>
       </c>
       <c r="D65" t="n" s="3">
-        <v>0.783</v>
+        <v>0.602</v>
       </c>
       <c r="E65" t="n" s="3">
-        <v>0.77</v>
+        <v>0.747</v>
       </c>
       <c r="F65" t="n" s="3">
-        <v>0.776</v>
+        <v>0.624</v>
       </c>
       <c r="G65" t="n" s="3">
-        <v>0.808</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="66">
@@ -1750,22 +1756,22 @@
         <v>43</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C66" t="n" s="3">
-        <v>0.708</v>
+        <v>0.789</v>
       </c>
       <c r="D66" t="n" s="3">
-        <v>0.637</v>
+        <v>0.738</v>
       </c>
       <c r="E66" t="n" s="3">
-        <v>0.79</v>
+        <v>0.753</v>
       </c>
       <c r="F66" t="n" s="3">
-        <v>0.674</v>
+        <v>0.744</v>
       </c>
       <c r="G66" t="n" s="3">
-        <v>0.708</v>
+        <v>0.789</v>
       </c>
     </row>
     <row r="67">
@@ -1773,22 +1779,68 @@
         <v>43</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C67" t="n" s="3">
-        <v>0.679</v>
+        <v>0.773</v>
       </c>
       <c r="D67" t="n" s="3">
-        <v>0.602</v>
+        <v>0.77</v>
       </c>
       <c r="E67" t="n" s="3">
-        <v>0.747</v>
+        <v>0.76</v>
       </c>
       <c r="F67" t="n" s="3">
-        <v>0.624</v>
+        <v>0.755</v>
       </c>
       <c r="G67" t="n" s="3">
-        <v>0.679</v>
+        <v>0.773</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B68" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="C68" t="n" s="3">
+        <v>0.812</v>
+      </c>
+      <c r="D68" t="n" s="3">
+        <v>0.798</v>
+      </c>
+      <c r="E68" t="n" s="3">
+        <v>0.79</v>
+      </c>
+      <c r="F68" t="n" s="3">
+        <v>0.789</v>
+      </c>
+      <c r="G68" t="n" s="3">
+        <v>0.812</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B69" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="C69" t="n" s="3">
+        <v>0.675</v>
+      </c>
+      <c r="D69" t="n" s="3">
+        <v>0.603</v>
+      </c>
+      <c r="E69" t="n" s="3">
+        <v>0.755</v>
+      </c>
+      <c r="F69" t="n" s="3">
+        <v>0.625</v>
+      </c>
+      <c r="G69" t="n" s="3">
+        <v>0.675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>